<commit_message>
docs: update zoho webhook spreadsheets
</commit_message>
<xml_diff>
--- a/docs/zoho-books-api-catalogue.xlsx
+++ b/docs/zoho-books-api-catalogue.xlsx
@@ -568,7 +568,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Prepared 2026-08-27  ·  Source: docs/zoho-books-api-usage.md  ·  Host: https://www.zohoapis.in/books/v3</t>
+          <t>Prepared 2026-08-31  ·  Source: docs/zoho-books-api-usage.md + shipment webhook deployment verification  ·  Host: https://www.zohoapis.in/books/v3</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F39"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1558,12 +1558,12 @@
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>Confirm sales-order state after create, or inspect a synced order in Zoho.</t>
+          <t>Confirm sales-order state after create; fallback source for tracking fields when webhook payload is incomplete.</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Order sync follow-up when we need the sales-order record; occasional status checks.</t>
+          <t>Order sync follow-up and tracking scheduler/admin fallback. Shipment webhook is now the primary event path on UAT.</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -1573,325 +1573,357 @@
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
-          <t>No per-API dollar charge and no pay-as-you-go overage. Exceeding the quota returns HTTP 429 (Zoho error code 45). Our pull stops cleanly and keeps what already saved. Extra volume is not sold; upgrade plan or request a limit increase from Zoho support. Light; not a high-volume catalog job.</t>
+          <t>No per-API dollar charge and no pay-as-you-go overage. Exceeding the quota returns HTTP 429 (Zoho error code 45). Shipment webhook reduces recurring tracking reads; keep this as fallback.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="78" customHeight="1">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
+          <t>GET /inventory/v1/packages?salesorder_number_contains={num}</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Zoho Inventory package lookup for a sales order number; returns package/shipment status, shipment id, AWB/carrier, and delivery state.</t>
+        </is>
+      </c>
+      <c r="C30" s="9" t="inlineStr">
+        <is>
+          <t>Fallback tracking pull for HAND_WRAPPED / shipped / delivered status when a webhook was missed or needs verification.</t>
+        </is>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Scheduler/admin pull-order-tracking fallback for CONFIRMED/HAND_WRAPPED Zoho-synced orders. Shipment webhook is live on UAT and should be the primary path.</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>Shared org quota; 1 Inventory API call per order checked when fallback runs.</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>No per-API dollar charge. Repeated scheduler fallback can burn quota; shipment webhook should avoid most recurring package reads.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="78" customHeight="1">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>PUT /salesorders/{id}/address/billing</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>One-off update of the sales-order billing address after create.</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>Apply the store billing address Zoho did not take on create.</t>
         </is>
       </c>
-      <c r="D30" s="8" t="inlineStr">
+      <c r="D31" s="8" t="inlineStr">
         <is>
           <t>Immediately after creating the sales order during paid order sync.</t>
         </is>
       </c>
-      <c r="E30" s="8" t="inlineStr">
+      <c r="E31" s="8" t="inlineStr">
         <is>
           <t>Shared org quota (not per-endpoint): 100 requests/minute. Daily: Free 1,000 | Standard 2,000 | Professional 5,000 | Premium/Elite/Ultimate 10,000. 1 call per order.</t>
         </is>
       </c>
-      <c r="F30" s="8" t="inlineStr">
+      <c r="F31" s="8" t="inlineStr">
         <is>
           <t>No per-API dollar charge and no pay-as-you-go overage. Exceeding the quota returns HTTP 429 (Zoho error code 45). Our pull stops cleanly and keeps what already saved. Extra volume is not sold; upgrade plan or request a limit increase from Zoho support. +1 of the ~6–10 calls per paid order.</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="78" customHeight="1">
-      <c r="A31" s="9" t="inlineStr">
+    <row r="32" ht="78" customHeight="1">
+      <c r="A32" s="9" t="inlineStr">
         <is>
           <t>PUT /salesorders/{id}/address/shipping</t>
         </is>
       </c>
-      <c r="B31" s="9" t="inlineStr">
+      <c r="B32" s="9" t="inlineStr">
         <is>
           <t>One-off update of the sales-order shipping address after create.</t>
         </is>
       </c>
-      <c r="C31" s="9" t="inlineStr">
+      <c r="C32" s="9" t="inlineStr">
         <is>
           <t>Apply the store shipping address Zoho did not take on create.</t>
         </is>
       </c>
-      <c r="D31" s="9" t="inlineStr">
+      <c r="D32" s="9" t="inlineStr">
         <is>
           <t>Immediately after creating the sales order during paid order sync.</t>
         </is>
       </c>
-      <c r="E31" s="9" t="inlineStr">
+      <c r="E32" s="9" t="inlineStr">
         <is>
           <t>Shared org quota (not per-endpoint): 100 requests/minute. Daily: Free 1,000 | Standard 2,000 | Professional 5,000 | Premium/Elite/Ultimate 10,000. 1 call per order.</t>
         </is>
       </c>
-      <c r="F31" s="9" t="inlineStr">
+      <c r="F32" s="9" t="inlineStr">
         <is>
           <t>No per-API dollar charge and no pay-as-you-go overage. Exceeding the quota returns HTTP 429 (Zoho error code 45). Our pull stops cleanly and keeps what already saved. Extra volume is not sold; upgrade plan or request a limit increase from Zoho support. +1 of the ~6–10 calls per paid order.</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="78" customHeight="1">
-      <c r="A32" s="8" t="inlineStr">
+    <row r="33" ht="78" customHeight="1">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>POST /salesorders/{id}/status/void</t>
         </is>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>Void a sales order in Books.</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
         <is>
           <t>Cancel / void the Zoho sales order when the Mini order must be reversed.</t>
         </is>
       </c>
-      <c r="D32" s="8" t="inlineStr">
+      <c r="D33" s="8" t="inlineStr">
         <is>
           <t>Order void / cancel path when a previously synced sales order must be voided.</t>
         </is>
       </c>
-      <c r="E32" s="8" t="inlineStr">
+      <c r="E33" s="8" t="inlineStr">
         <is>
           <t>Shared org quota (not per-endpoint): 100 requests/minute. Daily: Free 1,000 | Standard 2,000 | Professional 5,000 | Premium/Elite/Ultimate 10,000. 1 call per void.</t>
         </is>
       </c>
-      <c r="F32" s="8" t="inlineStr">
+      <c r="F33" s="8" t="inlineStr">
         <is>
           <t>No per-API dollar charge and no pay-as-you-go overage. Exceeding the quota returns HTTP 429 (Zoho error code 45). Our pull stops cleanly and keeps what already saved. Extra volume is not sold; upgrade plan or request a limit increase from Zoho support. Rare; only on void flows.</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="78" customHeight="1">
-      <c r="A33" s="9" t="inlineStr">
+    <row r="34" ht="78" customHeight="1">
+      <c r="A34" s="9" t="inlineStr">
         <is>
           <t>POST /invoices/fromsalesorder</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>Create an invoice from an existing sales order (salesorder_id query).</t>
         </is>
       </c>
-      <c r="C33" s="9" t="inlineStr">
+      <c r="C34" s="9" t="inlineStr">
         <is>
           <t>Bill the customer in Zoho after the sales order exists.</t>
         </is>
       </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="D34" s="9" t="inlineStr">
         <is>
           <t>Paid order sync, after sales order (and address updates).</t>
         </is>
       </c>
-      <c r="E33" s="9" t="inlineStr">
+      <c r="E34" s="9" t="inlineStr">
         <is>
           <t>Shared org quota (not per-endpoint): 100 requests/minute. Daily: Free 1,000 | Standard 2,000 | Professional 5,000 | Premium/Elite/Ultimate 10,000. 1 call per order.</t>
         </is>
       </c>
-      <c r="F33" s="9" t="inlineStr">
+      <c r="F34" s="9" t="inlineStr">
         <is>
           <t>No per-API dollar charge and no pay-as-you-go overage. Exceeding the quota returns HTTP 429 (Zoho error code 45). Our pull stops cleanly and keeps what already saved. Extra volume is not sold; upgrade plan or request a limit increase from Zoho support. Part of ~6–10 calls per paid order.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="78" customHeight="1">
-      <c r="A34" s="8" t="inlineStr">
+    <row r="35" ht="78" customHeight="1">
+      <c r="A35" s="8" t="inlineStr">
         <is>
           <t>GET /invoices/{id}</t>
         </is>
       </c>
-      <c r="B34" s="8" t="inlineStr">
+      <c r="B35" s="8" t="inlineStr">
         <is>
           <t>Read invoice details.</t>
         </is>
       </c>
-      <c r="C34" s="8" t="inlineStr">
+      <c r="C35" s="8" t="inlineStr">
         <is>
           <t>Confirm invoice state / fetch invoice fields after create or for PDF/status.</t>
         </is>
       </c>
-      <c r="D34" s="8" t="inlineStr">
+      <c r="D35" s="8" t="inlineStr">
         <is>
           <t>Order sync follow-up and invoice PDF / status checks.</t>
         </is>
       </c>
-      <c r="E34" s="8" t="inlineStr">
+      <c r="E35" s="8" t="inlineStr">
         <is>
           <t>Shared org quota (not per-endpoint): 100 requests/minute. Daily: Free 1,000 | Standard 2,000 | Professional 5,000 | Premium/Elite/Ultimate 10,000. 1 call per invoice.</t>
         </is>
       </c>
-      <c r="F34" s="8" t="inlineStr">
+      <c r="F35" s="8" t="inlineStr">
         <is>
           <t>No per-API dollar charge and no pay-as-you-go overage. Exceeding the quota returns HTTP 429 (Zoho error code 45). Our pull stops cleanly and keeps what already saved. Extra volume is not sold; upgrade plan or request a limit increase from Zoho support. Occasional extra call in order sync.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="78" customHeight="1">
-      <c r="A35" s="9" t="inlineStr">
+    <row r="36" ht="78" customHeight="1">
+      <c r="A36" s="9" t="inlineStr">
         <is>
           <t>POST /invoices/{id}/status/sent</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>Mark the invoice as sent.</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
+      <c r="C36" s="9" t="inlineStr">
         <is>
           <t>Move the invoice out of draft so it is treated as issued in Books.</t>
         </is>
       </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="D36" s="9" t="inlineStr">
         <is>
           <t>Paid order sync after invoice create.</t>
         </is>
       </c>
-      <c r="E35" s="9" t="inlineStr">
+      <c r="E36" s="9" t="inlineStr">
         <is>
           <t>Shared org quota (not per-endpoint): 100 requests/minute. Daily: Free 1,000 | Standard 2,000 | Professional 5,000 | Premium/Elite/Ultimate 10,000. 1 call per invoice.</t>
         </is>
       </c>
-      <c r="F35" s="9" t="inlineStr">
+      <c r="F36" s="9" t="inlineStr">
         <is>
           <t>No per-API dollar charge and no pay-as-you-go overage. Exceeding the quota returns HTTP 429 (Zoho error code 45). Our pull stops cleanly and keeps what already saved. Extra volume is not sold; upgrade plan or request a limit increase from Zoho support. Part of paid order sync.</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="78" customHeight="1">
-      <c r="A36" s="8" t="inlineStr">
+    <row r="37" ht="78" customHeight="1">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>POST /invoices/{id}/status/void</t>
         </is>
       </c>
-      <c r="B36" s="8" t="inlineStr">
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t>Void an invoice.</t>
         </is>
       </c>
-      <c r="C36" s="8" t="inlineStr">
+      <c r="C37" s="8" t="inlineStr">
         <is>
           <t>Reverse a synced invoice when the Mini order is voided/cancelled.</t>
         </is>
       </c>
-      <c r="D36" s="8" t="inlineStr">
+      <c r="D37" s="8" t="inlineStr">
         <is>
           <t>Order void path when an invoice was already created.</t>
         </is>
       </c>
-      <c r="E36" s="8" t="inlineStr">
+      <c r="E37" s="8" t="inlineStr">
         <is>
           <t>Shared org quota (not per-endpoint): 100 requests/minute. Daily: Free 1,000 | Standard 2,000 | Professional 5,000 | Premium/Elite/Ultimate 10,000. 1 call per void.</t>
         </is>
       </c>
-      <c r="F36" s="8" t="inlineStr">
+      <c r="F37" s="8" t="inlineStr">
         <is>
           <t>No per-API dollar charge and no pay-as-you-go overage. Exceeding the quota returns HTTP 429 (Zoho error code 45). Our pull stops cleanly and keeps what already saved. Extra volume is not sold; upgrade plan or request a limit increase from Zoho support. Rare; only on void flows.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="78" customHeight="1">
-      <c r="A37" s="9" t="inlineStr">
+    <row r="38" ht="78" customHeight="1">
+      <c r="A38" s="9" t="inlineStr">
         <is>
           <t>GET /invoices/pdf?invoice_ids={id}</t>
         </is>
       </c>
-      <c r="B37" s="9" t="inlineStr">
+      <c r="B38" s="9" t="inlineStr">
         <is>
           <t>Download invoice PDF binary.</t>
         </is>
       </c>
-      <c r="C37" s="9" t="inlineStr">
+      <c r="C38" s="9" t="inlineStr">
         <is>
           <t>Store / expose the Zoho invoice PDF on the Mini order.</t>
         </is>
       </c>
-      <c r="D37" s="9" t="inlineStr">
+      <c r="D38" s="9" t="inlineStr">
         <is>
           <t>After successful invoice create during order sync (when PDF fetch is enabled).</t>
         </is>
       </c>
-      <c r="E37" s="9" t="inlineStr">
+      <c r="E38" s="9" t="inlineStr">
         <is>
           <t>Shared org quota (not per-endpoint): 100 requests/minute. Daily: Free 1,000 | Standard 2,000 | Professional 5,000 | Premium/Elite/Ultimate 10,000. 1 call per PDF.</t>
         </is>
       </c>
-      <c r="F37" s="9" t="inlineStr">
+      <c r="F38" s="9" t="inlineStr">
         <is>
           <t>No per-API dollar charge and no pay-as-you-go overage. Exceeding the quota returns HTTP 429 (Zoho error code 45). Our pull stops cleanly and keeps what already saved. Extra volume is not sold; upgrade plan or request a limit increase from Zoho support. +1 call per synced order if PDF is fetched.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="78" customHeight="1">
-      <c r="A38" s="8" t="inlineStr">
+    <row r="39" ht="78" customHeight="1">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>POST /customerpayments</t>
         </is>
       </c>
-      <c r="B38" s="8" t="inlineStr">
+      <c r="B39" s="8" t="inlineStr">
         <is>
           <t>Record a customer payment against the invoice.</t>
         </is>
       </c>
-      <c r="C38" s="8" t="inlineStr">
+      <c r="C39" s="8" t="inlineStr">
         <is>
           <t>Mark the Zoho invoice paid to match the store payment.</t>
         </is>
       </c>
-      <c r="D38" s="8" t="inlineStr">
+      <c r="D39" s="8" t="inlineStr">
         <is>
           <t>Paid order sync after invoice is created/sent.</t>
         </is>
       </c>
-      <c r="E38" s="8" t="inlineStr">
+      <c r="E39" s="8" t="inlineStr">
         <is>
           <t>Shared org quota (not per-endpoint): 100 requests/minute. Daily: Free 1,000 | Standard 2,000 | Professional 5,000 | Premium/Elite/Ultimate 10,000. 1 call per payment.</t>
         </is>
       </c>
-      <c r="F38" s="8" t="inlineStr">
+      <c r="F39" s="8" t="inlineStr">
         <is>
           <t>No per-API dollar charge and no pay-as-you-go overage. Exceeding the quota returns HTTP 429 (Zoho error code 45). Our pull stops cleanly and keeps what already saved. Extra volume is not sold; upgrade plan or request a limit increase from Zoho support. Part of paid order sync.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="78" customHeight="1">
-      <c r="A39" s="9" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
         <is>
           <t>POST /inventoryadjustments</t>
         </is>
       </c>
-      <c r="B39" s="9" t="inlineStr">
+      <c r="B40" s="9" t="inlineStr">
         <is>
           <t>Create an inventory adjustment (on-hand qty).</t>
         </is>
       </c>
-      <c r="C39" s="9" t="inlineStr">
+      <c r="C40" s="9" t="inlineStr">
         <is>
           <t>Adjust Zoho on-hand quantity when stock sync is enabled.</t>
         </is>
       </c>
-      <c r="D39" s="9" t="inlineStr">
+      <c r="D40" s="9" t="inlineStr">
         <is>
           <t>Product push / stock sync when inventory adjustment is turned on.</t>
         </is>
       </c>
-      <c r="E39" s="9" t="inlineStr">
+      <c r="E40" s="9" t="inlineStr">
         <is>
           <t>Shared org quota (not per-endpoint): 100 requests/minute. Daily: Free 1,000 | Standard 2,000 | Professional 5,000 | Premium/Elite/Ultimate 10,000. 1 call per adjustment.</t>
         </is>
       </c>
-      <c r="F39" s="9" t="inlineStr">
+      <c r="F40" s="9" t="inlineStr">
         <is>
           <t>No per-API dollar charge and no pay-as-you-go overage. Exceeding the quota returns HTTP 429 (Zoho error code 45). Our pull stops cleanly and keeps what already saved. Extra volume is not sold; upgrade plan or request a limit increase from Zoho support. Extra on stock-enabled pushes; keep stock sync scoped.</t>
         </is>
@@ -1922,7 +1954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2424,6 +2456,38 @@
       <c r="F17" s="9" t="inlineStr">
         <is>
           <t>No per-API dollar charge and no pay-as-you-go overage. Exceeding the quota returns HTTP 429 (Zoho error code 45). Our pull stops cleanly and keeps what already saved. Extra volume is not sold; upgrade plan or request a limit increase from Zoho support. Rank 4 per order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>POST /api/v1/admin/zoho/pull-order-tracking</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Fallback pull for eligible Zoho-synced orders to refresh package/shipment tracking fields.</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Backfill or recover missed shipment webhook events; verify delivery status when needed.</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Admin/manual use and scheduler fallback. Frontend order tracking no longer polls this path.</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>Consumes Zoho quota through GET /salesorders/{id} and GET /inventory/v1/packages per order checked.</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>No per-API dollar charge. Use sparingly now that shipment webhook is deployed.</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2666,6 +2730,38 @@
       <c r="F8" s="12" t="inlineStr">
         <is>
           <t>No per-API dollar charge and no pay-as-you-go overage. Exceeding the quota returns HTTP 429 (Zoho error code 45). Our pull stops cleanly and keeps what already saved. Extra volume is not sold; upgrade plan or request a limit increase from Zoho support. Negligible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>5. Tracking fallback</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Checks eligible orders with sales-order/package GETs when webhook delivery needs fallback.</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>Keep store order tracking correct if Zoho workflow webhook misses an event.</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Scheduler/admin pull-order-tracking only; shipment webhook is primary on UAT. Frontend tracking API polling has been removed.</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>Roughly 1-2 calls per order checked when fallback runs.</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>Lower than catalog/order sync if kept sparse, but frequent scheduler polling wastes quota compared with the deployed shipment webhook.</t>
         </is>
       </c>
     </row>
@@ -2694,7 +2790,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -3164,6 +3260,38 @@
       <c r="F16" s="8" t="inlineStr">
         <is>
           <t>Lower than product pull because we skip per-SKU detail when possible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Typical: Tracking fallback for N orders</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>Sales-order/package reads for eligible orders when webhook backfill is needed.</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Fallback after shipment webhook deployment.</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Admin/manual or scheduler fallback, not browser polling.</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>≈ 1-2 calls × N orders checked.</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Keep interval sparse after Zoho Workflow Logs confirm webhook delivery.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add zoho item and order status webhooks
</commit_message>
<xml_diff>
--- a/docs/zoho-books-api-catalogue.xlsx
+++ b/docs/zoho-books-api-catalogue.xlsx
@@ -546,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:G17"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -558,6 +558,7 @@
     <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="28" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -568,10 +569,11 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Prepared 2026-08-31  ·  Source: docs/zoho-books-api-usage.md + shipment webhook deployment verification  ·  Host: https://www.zohoapis.in/books/v3</t>
-        </is>
-      </c>
-    </row>
+          <t>Prepared 2026-08-31  ·  Source: docs/zoho-books-api-usage.md + UAT webhook deployment verification  ·  Host: https://www.zohoapis.in/books/v3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -646,6 +648,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="B16" s="3" t="inlineStr">
         <is>
@@ -1083,7 +1086,7 @@
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Every SKU returned by a product pull (full or incremental). Also when we need a fresh item after create/update.</t>
+          <t>Single item pull from admin/manual import and item webhook. No full catalog scan needed for webhook events.</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
@@ -1563,7 +1566,7 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>Order sync follow-up and tracking scheduler/admin fallback. Shipment webhook is now the primary event path on UAT.</t>
+          <t>Order sync follow-up and sparse tracking fallback. Shipment and order-status webhooks are now primary on UAT.</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -1954,7 +1957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2488,6 +2491,70 @@
       <c r="F18" s="9" t="inlineStr">
         <is>
           <t>No per-API dollar charge. Use sparingly now that shipment webhook is deployed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>POST /api/v1/zoho/item-webhook</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Public Zoho webhook endpoint for item/catalog events.</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Runs single-item Zoho pull/merge by item_id or SKU; persists idempotency event.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Zoho Item Created/Edited workflow.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Consumes at most targeted item lookup/detail calls, not catalog pagination.</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>No per-endpoint charge; replaces broad catalog polling for changed rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>POST /api/v1/zoho/order-status-webhook</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Public Zoho webhook endpoint for sales-order status/void events.</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Updates local order status/tracking fields; void maps to CANCELLED.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Zoho Sales Order status/void workflow.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Avoids sales-order GET for void detection; fallback pulls remain available.</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>No per-endpoint charge; verify delivery in Zoho Workflow Logs.</t>
         </is>
       </c>
     </row>
@@ -2746,12 +2813,12 @@
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>Keep store order tracking correct if Zoho workflow webhook misses an event.</t>
+          <t>Recovery path if shipment or order-status webhook delivery is missed.</t>
         </is>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
-          <t>Scheduler/admin pull-order-tracking only; shipment webhook is primary on UAT. Frontend tracking API polling has been removed.</t>
+          <t>Scheduler/admin pull-order-tracking only; shipment and order-status webhooks are primary on UAT. Frontend tracking API polling has been removed.</t>
         </is>
       </c>
       <c r="E9" s="12" t="inlineStr">
@@ -3276,7 +3343,7 @@
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>Fallback after shipment webhook deployment.</t>
+          <t>Fallback after shipment/order-status webhook deployment.</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
@@ -3286,7 +3353,7 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t>≈ 1-2 calls × N orders checked.</t>
+          <t>Keep interval sparse after Zoho Workflow Logs confirm webhook delivery.</t>
         </is>
       </c>
       <c r="F17" s="8" t="inlineStr">

</xml_diff>